<commit_message>
Fix quantitative analysis inconsistencies
- results.tex: correct source-type breakdown from 6/4/4/3 to 4/3/4/6
- methods.tex: fix search date range from Jan 2015 to 2003; add rationale
- abstract.tex: update date range to 2003 onwards
- evidence_extraction_table.csv: S16 HIPAA year 2012 -> 2024
- prisma-counts.xlsx: fix subcategory counts, source names, exclusion note
</commit_message>
<xml_diff>
--- a/prisma/prisma-counts.xlsx
+++ b/prisma/prisma-counts.xlsx
@@ -1080,7 +1080,7 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Excl. reasons: wrong focus (~8); wrong outcome (~4); wrong setting (~3); narrative only (~3); duplicate of retained (~2); not retrievable (2) + 2 additional</t>
+          <t>Excl. reasons: wrong outcome (E2, n=9); insufficient methodology (E4, n=6); wrong setting (E3, n=4); duplicate/better source retained (E5, n=4); wrong focus (E1, n=1). See Supplementary File S2 for full list.</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>17 sources: 6 systematic/umbrella reviews; 4 scoping/narrative reviews; 4 government/audit reports; 3 policy/framework/theory analyses</t>
+          <t>17 sources: 4 systematic/umbrella reviews; 3 scoping/narrative reviews; 4 government/audit reports; 6 policy/regulatory/framework analyses</t>
         </is>
       </c>
     </row>
@@ -1119,12 +1119,12 @@
         </is>
       </c>
       <c r="B26" s="17" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C26" s="17" t="n"/>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>Holmes, Kruse, Fennelly, Aguirre, Bitar + 1 additional</t>
+          <t>Eden, Kruse, Fennelly, Torab-Miandoab</t>
         </is>
       </c>
     </row>
@@ -1135,12 +1135,12 @@
         </is>
       </c>
       <c r="B27" s="17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C27" s="17" t="n"/>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>Aguirre scoping, Adams qualitative case + 2 scoping reviews</t>
+          <t>Aguirre, Adams, DeLone &amp; McLean</t>
         </is>
       </c>
     </row>
@@ -1163,16 +1163,16 @@
     <row r="29" ht="38" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  → Policy / framework / theory</t>
+          <t xml:space="preserve">  → Policy / regulatory / framework analyses</t>
         </is>
       </c>
       <c r="B29" s="17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C29" s="17" t="n"/>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>EU/Estonia EHR Law; NIST 800-37 &amp; 800-53; HIPAA De-id; DeLone &amp; McLean IS</t>
+          <t>Holmgren (2023); Estonia eHealth System (2026); EU/Estonia EHR Law (2016); NIST SP 800-37 (2018); NIST SP 800-53 (2020); HIPAA De-identification (2024)</t>
         </is>
       </c>
     </row>

</xml_diff>